<commit_message>
+Code pour pilotage du DAC121S101_Driver.vhd par code python
</commit_message>
<xml_diff>
--- a/doc/IO.xlsx
+++ b/doc/IO.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\3Utransat\TUT_EGSE_EP_ADS7049\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\3Utransat\TUT_EGSE_EP_ads7049_branch\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9384"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9390"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
   <si>
     <t>FPGA PIN</t>
   </si>
@@ -108,6 +108,57 @@
   </si>
   <si>
     <t xml:space="preserve">IO_L14P_T2_SRCC_34 </t>
+  </si>
+  <si>
+    <t>o_DAC_SCLK</t>
+  </si>
+  <si>
+    <t>o_DAC_SYNC_n</t>
+  </si>
+  <si>
+    <t>o_DAC_DIN</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>F3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J4-11 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">J4-12 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">J4-13 </t>
+  </si>
+  <si>
+    <t>L5</t>
+  </si>
+  <si>
+    <t>N3</t>
+  </si>
+  <si>
+    <t>N4</t>
+  </si>
+  <si>
+    <t>J3-21</t>
+  </si>
+  <si>
+    <t>J3-23</t>
+  </si>
+  <si>
+    <t>J3-19</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>no test</t>
   </si>
 </sst>
 </file>
@@ -428,17 +479,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.109375" customWidth="1"/>
-    <col min="3" max="3" width="27.77734375" customWidth="1"/>
-    <col min="4" max="4" width="19.88671875" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" customWidth="1"/>
-    <col min="6" max="6" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -458,7 +509,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -477,8 +528,11 @@
       <c r="F2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -497,8 +551,11 @@
       <c r="F3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -511,8 +568,11 @@
       <c r="F4" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -525,8 +585,11 @@
       <c r="F5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -538,6 +601,93 @@
       </c>
       <c r="F6" t="s">
         <v>26</v>
+      </c>
+      <c r="G6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" t="s">
+        <v>40</v>
+      </c>
+      <c r="G12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Première version avec controle saturante dans energy_level.vhd conditionné sur "i_data_before_filter" TH_ADC wire 07, + Correction dans spectrum_FSM.vhd dans l'état "end_write_to_gse" afin d'assuré un raz de l'add 1023 de la RAM
</commit_message>
<xml_diff>
--- a/doc/IO.xlsx
+++ b/doc/IO.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="45">
   <si>
     <t>FPGA PIN</t>
   </si>
@@ -479,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" customWidth="1"/>
@@ -690,6 +690,48 @@
         <v>43</v>
       </c>
     </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16" t="s">
+        <v>40</v>
+      </c>
+      <c r="G16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" t="s">
+        <v>42</v>
+      </c>
+      <c r="G17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18" t="s">
+        <v>41</v>
+      </c>
+      <c r="G18" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>